<commit_message>
Update README and figure scripts
</commit_message>
<xml_diff>
--- a/Preliminary data/database_unique_references.xlsx
+++ b/Preliminary data/database_unique_references.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hounkpk1\RAP_Drivers\output\Figure_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hounkpk1\RAP_Drivers\Preliminary data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68DDD04-862D-46A0-AEF4-08522E36B721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FB4D31-2721-483C-BA00-B7747D2B85A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2483" uniqueCount="1633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="1632">
   <si>
     <t>references</t>
   </si>
@@ -4892,9 +4892,6 @@
   </si>
   <si>
     <t>wang x nutrent restoraton effects and water erosion percentation and control of slope farmland of conservative tillage loess plateau in northern shaanxi northwest af university 2013</t>
-  </si>
-  <si>
-    <t>PhD</t>
   </si>
   <si>
     <t>Xia, Longlong, Shu Kee Lam, Xiaoyuan Yan, and Deli Chen. "How does recycling of livestock manure in agroecosystems affect crop productivity, reactive nitrogen losses, and soil carbon balance?." Environmental Science &amp; Technology 51, no. 13 (2017): 7450-7457.</t>
@@ -15158,19 +15155,16 @@
       <c r="D494" s="2">
         <v>2013</v>
       </c>
-      <c r="E494" s="2" t="s">
-        <v>1624</v>
-      </c>
       <c r="F494" s="2" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="495" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A495" s="2" t="s">
+        <v>1624</v>
+      </c>
+      <c r="B495" s="2" t="s">
         <v>1625</v>
-      </c>
-      <c r="B495" s="2" t="s">
-        <v>1626</v>
       </c>
       <c r="D495" s="2">
         <v>2017</v>
@@ -15181,10 +15175,10 @@
     </row>
     <row r="496" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A496" s="2" t="s">
+        <v>1626</v>
+      </c>
+      <c r="B496" s="2" t="s">
         <v>1627</v>
-      </c>
-      <c r="B496" s="2" t="s">
-        <v>1628</v>
       </c>
       <c r="D496" s="2">
         <v>2018</v>
@@ -15195,10 +15189,10 @@
     </row>
     <row r="497" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A497" s="2" t="s">
+        <v>1628</v>
+      </c>
+      <c r="B497" s="2" t="s">
         <v>1629</v>
-      </c>
-      <c r="B497" s="2" t="s">
-        <v>1630</v>
       </c>
       <c r="D497" s="2">
         <v>2018</v>
@@ -15209,10 +15203,10 @@
     </row>
     <row r="498" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A498" s="2" t="s">
+        <v>1630</v>
+      </c>
+      <c r="B498" s="2" t="s">
         <v>1631</v>
-      </c>
-      <c r="B498" s="2" t="s">
-        <v>1632</v>
       </c>
       <c r="D498" s="2">
         <v>2017</v>

</xml_diff>